<commit_message>
Improve AdSense content, preserve traffic pages, and split blog bundles
</commit_message>
<xml_diff>
--- a/public/samples/youtube-playlist-export-sample.xlsx
+++ b/public/samples/youtube-playlist-export-sample.xlsx
@@ -79,10 +79,10 @@
     <t>Example Channel</t>
   </si>
   <si>
-    <t>00:12:34</t>
-  </si>
-  <si>
-    <t>12 minutes, 34 seconds</t>
+    <t>12:34</t>
+  </si>
+  <si>
+    <t>12 Minutes, 34 Seconds</t>
   </si>
   <si>
     <t>2026-01-15T10:30:00</t>
@@ -112,10 +112,10 @@
     <t>https://i.ytimg.com/vi/VIDEO_ID_02/hqdefault.jpg</t>
   </si>
   <si>
-    <t>00:04:05</t>
-  </si>
-  <si>
-    <t>4 minutes, 5 seconds</t>
+    <t>4:05</t>
+  </si>
+  <si>
+    <t>4 Minutes, 5 Seconds</t>
   </si>
   <si>
     <t>2026-02-20T08:00:00</t>

</xml_diff>